<commit_message>
Leave a gap column before the weekly audit pivot and drop Count of Amount
The Processed sheet's data table ends at column G (Source date), and the
Category pivot started right next to it in H. Move the pivot and its "Pivot
Table" label to column I so column H stays empty, and remove the Count of
Amount value so the pivot shows only Category and Sum of Amount. Applies to
both the GTO and Creator Club templates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKca3uHMgVXE6K4VFiS7ma
</commit_message>
<xml_diff>
--- a/api/templates/creator_weekly_audit_base.xlsx
+++ b/api/templates/creator_weekly_audit_base.xlsx
@@ -179,7 +179,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="CategoryPivot" cacheId="0" dataCaption="Values" compact="0" compactData="0">
-  <location ref="H2:J3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="I2:J3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -200,15 +200,11 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
   <colItems count="1">
     <i/>
   </colItems>
-  <dataFields count="2">
+  <dataFields count="1">
     <dataField name="Sum of Amount" fld="2" baseField="0" baseItem="0"/>
-    <dataField name="Count of Amount" fld="2" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
 </pivotTableDefinition>
 </file>
@@ -517,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,7 +547,7 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Pivot Table</t>
         </is>

</xml_diff>